<commit_message>
fix: fixed faulty validation code
</commit_message>
<xml_diff>
--- a/src/test_xlsx/oddi-test.xlsx
+++ b/src/test_xlsx/oddi-test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SBC\oddiville-proj\oddiville-frontend\src\test_xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FF28150-415A-4A11-A1DB-8FA85C918C89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E794E83-0ED9-46FE-B0AE-9763514C3D8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3810" yWindow="3810" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="660" yWindow="3735" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t>item</t>
   </si>
@@ -571,9 +571,7 @@
       <c r="F4" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G4" s="2">
-        <v>1100</v>
-      </c>
+      <c r="G4" s="2"/>
       <c r="H4" s="2" t="s">
         <v>27</v>
       </c>
@@ -612,9 +610,7 @@
       <c r="E5" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="F5" s="2" t="s">
-        <v>16</v>
-      </c>
+      <c r="F5" s="2"/>
       <c r="G5" s="2">
         <v>1700</v>
       </c>
@@ -642,5 +638,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: added file requirement validation and added toasts for onscreen notifications
</commit_message>
<xml_diff>
--- a/src/test_xlsx/oddi-test.xlsx
+++ b/src/test_xlsx/oddi-test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SBC\oddiville-proj\oddiville-frontend\src\test_xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E794E83-0ED9-46FE-B0AE-9763514C3D8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4DBE5FE-CD6C-4CDF-A092-4E44B413FAB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="660" yWindow="3735" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3810" yWindow="3810" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="33">
   <si>
     <t>item</t>
   </si>
@@ -571,7 +571,9 @@
       <c r="F4" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G4" s="2"/>
+      <c r="G4" s="2">
+        <v>1100</v>
+      </c>
       <c r="H4" s="2" t="s">
         <v>27</v>
       </c>
@@ -610,7 +612,9 @@
       <c r="E5" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="F5" s="2"/>
+      <c r="F5" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="G5" s="2">
         <v>1700</v>
       </c>

</xml_diff>